<commit_message>
Rename Grinds to Grind (matches storefront)
Visible copy, nav, /grind route (old /grinds redirects), page title,
manifest, and link preview image. Internal keys unchanged so the live
sheet keeps working; hours accept shop 'grind' or 'grinds'.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/sheet-template/Grumpy Goat Website Content.xlsx
+++ b/sheet-template/Grumpy Goat Website Content.xlsx
@@ -622,7 +622,7 @@
       </c>
       <c r="B3" s="5" t="inlineStr">
         <is>
-          <t>Gear &amp; Grinds</t>
+          <t>Gear &amp; Grind</t>
         </is>
       </c>
       <c r="C3" s="6" t="inlineStr">
@@ -1030,7 +1030,7 @@
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>Grumpy Goat Grinds</t>
+          <t>Grumpy Goat Grind</t>
         </is>
       </c>
       <c r="C27" s="6" t="inlineStr">
@@ -1370,7 +1370,7 @@
       </c>
       <c r="B47" s="5" t="inlineStr">
         <is>
-          <t>Grumpy Goat Grinds</t>
+          <t>Grumpy Goat Grind</t>
         </is>
       </c>
       <c r="C47" s="6" t="inlineStr">
@@ -1506,7 +1506,7 @@
       </c>
       <c r="B55" s="5" t="inlineStr">
         <is>
-          <t>Settle into a booth, catch the race on the big screen, or sprawl out on the couch with your dog. Grumpy Goat Grinds is built for hanging out — because the best part of the ride is the stories after.</t>
+          <t>Settle into a booth, catch the race on the big screen, or sprawl out on the couch with your dog. Grumpy Goat Grind is built for hanging out — because the best part of the ride is the stories after.</t>
         </is>
       </c>
       <c r="C55" s="6" t="inlineStr">
@@ -1928,7 +1928,7 @@
     <row r="9">
       <c r="A9" s="7" t="inlineStr">
         <is>
-          <t>grinds</t>
+          <t>grind</t>
         </is>
       </c>
       <c r="B9" s="7" t="inlineStr">
@@ -1945,7 +1945,7 @@
     <row r="10">
       <c r="A10" s="7" t="inlineStr">
         <is>
-          <t>grinds</t>
+          <t>grind</t>
         </is>
       </c>
       <c r="B10" s="7" t="inlineStr">
@@ -1962,7 +1962,7 @@
     <row r="11">
       <c r="A11" s="7" t="inlineStr">
         <is>
-          <t>grinds</t>
+          <t>grind</t>
         </is>
       </c>
       <c r="B11" s="7" t="inlineStr">
@@ -1979,7 +1979,7 @@
     <row r="12">
       <c r="A12" s="7" t="inlineStr">
         <is>
-          <t>grinds</t>
+          <t>grind</t>
         </is>
       </c>
       <c r="B12" s="7" t="inlineStr">
@@ -1996,7 +1996,7 @@
     <row r="13">
       <c r="A13" s="7" t="inlineStr">
         <is>
-          <t>grinds</t>
+          <t>grind</t>
         </is>
       </c>
       <c r="B13" s="7" t="inlineStr">
@@ -2013,7 +2013,7 @@
     <row r="14">
       <c r="A14" s="7" t="inlineStr">
         <is>
-          <t>grinds</t>
+          <t>grind</t>
         </is>
       </c>
       <c r="B14" s="7" t="inlineStr">
@@ -2030,7 +2030,7 @@
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
         <is>
-          <t>grinds</t>
+          <t>grind</t>
         </is>
       </c>
       <c r="B15" s="7" t="inlineStr">

</xml_diff>

<commit_message>
Refactor internal grinds names to grind
Text keys (home.grind.*, grind.*, contact.grindHours), files, components,
and CSS classes. Sheet template regenerated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/sheet-template/Grumpy Goat Website Content.xlsx
+++ b/sheet-template/Grumpy Goat Website Content.xlsx
@@ -1025,7 +1025,7 @@
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
         <is>
-          <t>home.grinds.label</t>
+          <t>home.grind.label</t>
         </is>
       </c>
       <c r="B27" s="5" t="inlineStr">
@@ -1042,7 +1042,7 @@
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
         <is>
-          <t>home.grinds.title</t>
+          <t>home.grind.title</t>
         </is>
       </c>
       <c r="B28" s="5" t="inlineStr">
@@ -1059,7 +1059,7 @@
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
         <is>
-          <t>home.grinds.body</t>
+          <t>home.grind.body</t>
         </is>
       </c>
       <c r="B29" s="5" t="inlineStr">
@@ -1076,7 +1076,7 @@
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
         <is>
-          <t>home.grinds.feature1.title</t>
+          <t>home.grind.feature1.title</t>
         </is>
       </c>
       <c r="B30" s="5" t="inlineStr">
@@ -1093,7 +1093,7 @@
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
         <is>
-          <t>home.grinds.feature1.text</t>
+          <t>home.grind.feature1.text</t>
         </is>
       </c>
       <c r="B31" s="5" t="inlineStr">
@@ -1110,7 +1110,7 @@
     <row r="32">
       <c r="A32" s="4" t="inlineStr">
         <is>
-          <t>home.grinds.feature2.title</t>
+          <t>home.grind.feature2.title</t>
         </is>
       </c>
       <c r="B32" s="5" t="inlineStr">
@@ -1127,7 +1127,7 @@
     <row r="33">
       <c r="A33" s="4" t="inlineStr">
         <is>
-          <t>home.grinds.feature2.text</t>
+          <t>home.grind.feature2.text</t>
         </is>
       </c>
       <c r="B33" s="5" t="inlineStr">
@@ -1144,7 +1144,7 @@
     <row r="34">
       <c r="A34" s="4" t="inlineStr">
         <is>
-          <t>home.grinds.feature3.title</t>
+          <t>home.grind.feature3.title</t>
         </is>
       </c>
       <c r="B34" s="5" t="inlineStr">
@@ -1161,7 +1161,7 @@
     <row r="35">
       <c r="A35" s="4" t="inlineStr">
         <is>
-          <t>home.grinds.feature3.text</t>
+          <t>home.grind.feature3.text</t>
         </is>
       </c>
       <c r="B35" s="5" t="inlineStr">
@@ -1178,7 +1178,7 @@
     <row r="36">
       <c r="A36" s="4" t="inlineStr">
         <is>
-          <t>home.grinds.button</t>
+          <t>home.grind.button</t>
         </is>
       </c>
       <c r="B36" s="5" t="inlineStr">
@@ -1365,7 +1365,7 @@
     <row r="47">
       <c r="A47" s="4" t="inlineStr">
         <is>
-          <t>grinds.hero.title</t>
+          <t>grind.hero.title</t>
         </is>
       </c>
       <c r="B47" s="5" t="inlineStr">
@@ -1382,7 +1382,7 @@
     <row r="48">
       <c r="A48" s="4" t="inlineStr">
         <is>
-          <t>grinds.menu.title</t>
+          <t>grind.menu.title</t>
         </is>
       </c>
       <c r="B48" s="5" t="inlineStr">
@@ -1399,7 +1399,7 @@
     <row r="49">
       <c r="A49" s="4" t="inlineStr">
         <is>
-          <t>grinds.menu.subtitle</t>
+          <t>grind.menu.subtitle</t>
         </is>
       </c>
       <c r="B49" s="5" t="inlineStr">
@@ -1416,7 +1416,7 @@
     <row r="50">
       <c r="A50" s="4" t="inlineStr">
         <is>
-          <t>grinds.menu.hot</t>
+          <t>grind.menu.hot</t>
         </is>
       </c>
       <c r="B50" s="5" t="inlineStr">
@@ -1433,7 +1433,7 @@
     <row r="51">
       <c r="A51" s="4" t="inlineStr">
         <is>
-          <t>grinds.menu.cold</t>
+          <t>grind.menu.cold</t>
         </is>
       </c>
       <c r="B51" s="5" t="inlineStr">
@@ -1450,7 +1450,7 @@
     <row r="52">
       <c r="A52" s="4" t="inlineStr">
         <is>
-          <t>grinds.hours.title</t>
+          <t>grind.hours.title</t>
         </is>
       </c>
       <c r="B52" s="5" t="inlineStr">
@@ -1467,7 +1467,7 @@
     <row r="53">
       <c r="A53" s="4" t="inlineStr">
         <is>
-          <t>grinds.hours.subtitle</t>
+          <t>grind.hours.subtitle</t>
         </is>
       </c>
       <c r="B53" s="5" t="inlineStr">
@@ -1484,7 +1484,7 @@
     <row r="54">
       <c r="A54" s="4" t="inlineStr">
         <is>
-          <t>grinds.atmosphere.title</t>
+          <t>grind.atmosphere.title</t>
         </is>
       </c>
       <c r="B54" s="5" t="inlineStr">
@@ -1501,7 +1501,7 @@
     <row r="55">
       <c r="A55" s="4" t="inlineStr">
         <is>
-          <t>grinds.atmosphere.body</t>
+          <t>grind.atmosphere.body</t>
         </is>
       </c>
       <c r="B55" s="5" t="inlineStr">
@@ -1705,7 +1705,7 @@
     <row r="67">
       <c r="A67" s="4" t="inlineStr">
         <is>
-          <t>contact.grindsHours</t>
+          <t>contact.grindHours</t>
         </is>
       </c>
       <c r="B67" s="5" t="inlineStr">

</xml_diff>